<commit_message>
cambios en ARCAT 09.04.2026
</commit_message>
<xml_diff>
--- a/00000_Correcciones/Cohorte06_TP01/Cohoorte06.xlsx
+++ b/00000_Correcciones/Cohorte06_TP01/Cohoorte06.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\00_ENGITHUB\Modulo02_JavaScript\00000_Correcciones\Cohorte06_TP01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E11C6E87-EB32-47B2-9DCC-B51418F6EC22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2417132C-ACDA-4334-81F0-6FBC39CDBE2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32415" yWindow="3285" windowWidth="21600" windowHeight="12690" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30855" yWindow="3705" windowWidth="21600" windowHeight="12690" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="66">
   <si>
     <t>Acosta Nieva, Nicole Nazarena</t>
   </si>
@@ -208,6 +208,21 @@
   </si>
   <si>
     <t>Bazán, Oscar Alfredo</t>
+  </si>
+  <si>
+    <t>Herrera, Mario Alberto</t>
+  </si>
+  <si>
+    <t>Maidana, Alejo Leonel</t>
+  </si>
+  <si>
+    <t>Monges, Braian</t>
+  </si>
+  <si>
+    <t>Cirione Leguizamon, Erik Mirko</t>
+  </si>
+  <si>
+    <t>Cano, Marcelo Emanuel</t>
   </si>
 </sst>
 </file>
@@ -279,10 +294,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -563,7 +578,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:G53"/>
+  <dimension ref="B2:G58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="7.28515625" bestFit="1" customWidth="1"/>
@@ -575,14 +590,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
@@ -1051,20 +1066,20 @@
       </c>
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B34" s="4">
+      <c r="B34" s="3">
         <v>31</v>
       </c>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4" t="s">
+      <c r="C34" s="3"/>
+      <c r="D34" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E34" s="4" t="s">
+      <c r="E34" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F34" s="4">
-        <v>2</v>
-      </c>
-      <c r="G34" s="4" t="s">
+      <c r="F34" s="3">
+        <v>2</v>
+      </c>
+      <c r="G34" s="3" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1237,22 +1252,22 @@
       </c>
     </row>
     <row r="47" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B47" s="4">
+      <c r="B47" s="3">
         <v>44</v>
       </c>
-      <c r="C47" s="4" t="s">
+      <c r="C47" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="D47" s="4" t="s">
+      <c r="D47" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E47" s="4" t="s">
+      <c r="E47" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F47" s="4">
-        <v>2</v>
-      </c>
-      <c r="G47" s="4" t="s">
+      <c r="F47" s="3">
+        <v>2</v>
+      </c>
+      <c r="G47" s="3" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1337,6 +1352,76 @@
         <v>2</v>
       </c>
       <c r="F53">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B54">
+        <v>51</v>
+      </c>
+      <c r="D54" t="s">
+        <v>61</v>
+      </c>
+      <c r="E54" t="s">
+        <v>2</v>
+      </c>
+      <c r="F54">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B55">
+        <v>52</v>
+      </c>
+      <c r="D55" t="s">
+        <v>62</v>
+      </c>
+      <c r="E55" t="s">
+        <v>2</v>
+      </c>
+      <c r="F55">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B56">
+        <v>53</v>
+      </c>
+      <c r="D56" t="s">
+        <v>63</v>
+      </c>
+      <c r="E56" t="s">
+        <v>2</v>
+      </c>
+      <c r="F56">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="57" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B57">
+        <v>54</v>
+      </c>
+      <c r="D57" t="s">
+        <v>64</v>
+      </c>
+      <c r="E57" t="s">
+        <v>2</v>
+      </c>
+      <c r="F57">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="58" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B58">
+        <v>55</v>
+      </c>
+      <c r="D58" t="s">
+        <v>65</v>
+      </c>
+      <c r="E58" t="s">
+        <v>2</v>
+      </c>
+      <c r="F58">
         <v>8</v>
       </c>
     </row>

</xml_diff>